<commit_message>
add scatter_3d for the drugs_allocated.
</commit_message>
<xml_diff>
--- a/static/allocate.xlsx
+++ b/static/allocate.xlsx
@@ -64,10 +64,10 @@
     <t>12月</t>
   </si>
   <si>
-    <t>品項總計</t>
-  </si>
-  <si>
-    <t>備註及可能原因</t>
+    <t>調撥總計</t>
+  </si>
+  <si>
+    <t>備註</t>
   </si>
   <si>
     <t>3MA01E</t>
@@ -77758,7 +77758,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="34" operator="greaterThanOrEqual" id="{007300DD-0019-49AA-AED7-005A008500A9}">
+          <x14:cfRule type="cellIs" priority="34" operator="greaterThanOrEqual" id="{002E007C-007F-417F-B736-008F00B70051}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <fill>

</xml_diff>